<commit_message>
rapeseed cake instead of meal in organic rations in BroilerHerd, LayerHerd and SheepHerd
</commit_message>
<xml_diff>
--- a/data/default/BroilerHerd.xlsx
+++ b/data/default/BroilerHerd.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\prod_parameters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="130">
   <si>
     <t>Höns</t>
   </si>
@@ -404,6 +404,18 @@
   </si>
   <si>
     <t>???</t>
+  </si>
+  <si>
+    <t>organic</t>
+  </si>
+  <si>
+    <t>conventional</t>
+  </si>
+  <si>
+    <t>rapeseed cake for organic rations</t>
+  </si>
+  <si>
+    <t>rapeseed cake</t>
   </si>
 </sst>
 </file>
@@ -413,7 +425,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -459,6 +471,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="7"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-9.9978637043366805E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -499,7 +531,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -522,6 +554,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -968,7 +1003,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="15.7109375" customWidth="1"/>
@@ -1417,7 +1452,7 @@
         <v>4.8486932599724906</v>
       </c>
     </row>
-    <row r="33" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
         <v>85</v>
       </c>
@@ -1428,7 +1463,7 @@
         <v>2.9917469050894088</v>
       </c>
     </row>
-    <row r="34" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C34" t="s">
         <v>86</v>
       </c>
@@ -1439,7 +1474,7 @@
         <v>6.5064269790826748</v>
       </c>
     </row>
-    <row r="35" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C35" t="s">
         <v>87</v>
       </c>
@@ -1450,7 +1485,10 @@
         <v>18.569463548830814</v>
       </c>
     </row>
-    <row r="36" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>127</v>
+      </c>
       <c r="C36" t="s">
         <v>88</v>
       </c>
@@ -1461,53 +1499,72 @@
         <v>2.9881895365934641</v>
       </c>
     </row>
-    <row r="37" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C37" t="s">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="D37" s="19" t="str">
+        <f>D36</f>
+        <v>share_in_ration</v>
+      </c>
+      <c r="E37" s="20">
+        <f>E36</f>
+        <v>2.9881895365934641</v>
+      </c>
+      <c r="G37" s="18" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
         <v>89</v>
-      </c>
-      <c r="D37" t="s">
-        <v>81</v>
-      </c>
-      <c r="E37" s="11">
-        <v>0.64032632927002808</v>
-      </c>
-    </row>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C38" t="s">
-        <v>98</v>
       </c>
       <c r="D38" t="s">
         <v>81</v>
       </c>
       <c r="E38" s="11">
-        <v>2.7854195323246222</v>
-      </c>
-    </row>
-    <row r="39" spans="3:7" x14ac:dyDescent="0.25">
+        <v>0.64032632927002808</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C39" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="D39" t="s">
         <v>81</v>
       </c>
       <c r="E39" s="11">
+        <v>2.7854195323246222</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C40" t="s">
+        <v>90</v>
+      </c>
+      <c r="D40" t="s">
+        <v>81</v>
+      </c>
+      <c r="E40" s="11">
         <v>1.66010529810748</v>
       </c>
-      <c r="G39" s="15" t="s">
+      <c r="G40" s="15" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="40" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C40" s="15" t="s">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C41" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="E40" s="11"/>
-    </row>
-    <row r="41" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C41" s="15" t="s">
+      <c r="E41" s="11"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C42" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="E41" s="11"/>
+      <c r="E42" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added live weight of lost animals for broilers
</commit_message>
<xml_diff>
--- a/data/default/BroilerHerd.xlsx
+++ b/data/default/BroilerHerd.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="131">
   <si>
     <t>Höns</t>
   </si>
@@ -403,9 +403,6 @@
     <t>Statistics Netherlands (2012)</t>
   </si>
   <si>
-    <t>???</t>
-  </si>
-  <si>
     <t>organic</t>
   </si>
   <si>
@@ -416,6 +413,12 @@
   </si>
   <si>
     <t>rapeseed cake</t>
+  </si>
+  <si>
+    <t>Clune et al. (2017)</t>
+  </si>
+  <si>
+    <t>kg LW/kg CW</t>
   </si>
 </sst>
 </file>
@@ -1329,10 +1332,10 @@
         <v>1.4285714285714286</v>
       </c>
       <c r="F22" t="s">
-        <v>57</v>
+        <v>130</v>
       </c>
       <c r="H22" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -1487,7 +1490,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C36" t="s">
         <v>88</v>
@@ -1501,10 +1504,10 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="19" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C37" s="18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D37" s="19" t="str">
         <f>D36</f>
@@ -1515,7 +1518,7 @@
         <v>2.9881895365934641</v>
       </c>
       <c r="G37" s="18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>